<commit_message>
chore: regenerate review sheets with full C-candidate wayback coverage
wayback --resume looked up 713 URLs (390 C-candidate blanks, 301 stuck
api_error_429 rows, 2 timeouts, plus new dead-URL coverage). Every
wayback row now has a final status: 2253 found / 1037 not_archived.

Rebrand verdicts unchanged (147 probably-broken / 293 probably-fine /
60 needs-human). Downstream shifts:
- probably-broken C-candidates: 102 now salvage-wayback (was 0),
  38 remove-or-replace (was 140), 7 bulk-unlink
- pages sheet: delete-page-candidate 229 -> 169,
  salvage-wayback 286 -> 346, fix-links-only 691 unchanged

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/utils/link_review_pages.xlsx
+++ b/utils/link_review_pages.xlsx
@@ -591,10 +591,10 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -659,10 +659,10 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -795,10 +795,10 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1271,10 +1271,10 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1543,10 +1543,10 @@
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -1611,10 +1611,10 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -1679,10 +1679,10 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -3163,10 +3163,10 @@
         <v>2</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q40" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
@@ -4123,10 +4123,10 @@
         <v>0</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
@@ -8603,10 +8603,10 @@
         <v>0</v>
       </c>
       <c r="P125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R125" t="inlineStr">
         <is>
@@ -9051,10 +9051,10 @@
         <v>0</v>
       </c>
       <c r="P132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R132" t="inlineStr">
         <is>
@@ -10011,10 +10011,10 @@
         <v>3</v>
       </c>
       <c r="P147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q147" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R147" t="inlineStr">
         <is>
@@ -11099,10 +11099,10 @@
         <v>6</v>
       </c>
       <c r="P164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q164" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R164" t="inlineStr">
         <is>
@@ -11675,10 +11675,10 @@
         <v>4</v>
       </c>
       <c r="P173" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q173" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R173" t="inlineStr">
         <is>
@@ -12059,10 +12059,10 @@
         <v>5</v>
       </c>
       <c r="P179" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q179" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R179" t="inlineStr">
         <is>
@@ -13275,10 +13275,10 @@
         <v>0</v>
       </c>
       <c r="P198" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q198" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R198" t="inlineStr">
         <is>
@@ -13659,10 +13659,10 @@
         <v>0</v>
       </c>
       <c r="P204" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q204" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R204" t="inlineStr">
         <is>
@@ -13979,10 +13979,10 @@
         <v>0</v>
       </c>
       <c r="P209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q209" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R209" t="inlineStr">
         <is>
@@ -15131,10 +15131,10 @@
         <v>9</v>
       </c>
       <c r="P227" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q227" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R227" t="inlineStr">
         <is>
@@ -18115,10 +18115,10 @@
         <v>0</v>
       </c>
       <c r="P272" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q272" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R272" t="inlineStr">
         <is>
@@ -18319,10 +18319,10 @@
         <v>0</v>
       </c>
       <c r="P275" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q275" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R275" t="inlineStr">
         <is>
@@ -18387,10 +18387,10 @@
         <v>0</v>
       </c>
       <c r="P276" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q276" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R276" t="inlineStr">
         <is>
@@ -18591,10 +18591,10 @@
         <v>0</v>
       </c>
       <c r="P279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q279" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R279" t="inlineStr">
         <is>
@@ -18727,10 +18727,10 @@
         <v>0</v>
       </c>
       <c r="P281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q281" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R281" t="inlineStr">
         <is>
@@ -18863,10 +18863,10 @@
         <v>0</v>
       </c>
       <c r="P283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q283" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R283" t="inlineStr">
         <is>
@@ -19271,10 +19271,10 @@
         <v>3</v>
       </c>
       <c r="P289" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q289" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R289" t="inlineStr">
         <is>
@@ -20155,10 +20155,10 @@
         <v>5</v>
       </c>
       <c r="P302" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q302" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R302" t="inlineStr">
         <is>
@@ -24167,10 +24167,10 @@
         <v>0</v>
       </c>
       <c r="P361" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q361" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R361" t="inlineStr">
         <is>
@@ -24439,14 +24439,14 @@
         <v>0</v>
       </c>
       <c r="P365" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q365" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R365" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -24507,14 +24507,14 @@
         <v>0</v>
       </c>
       <c r="P366" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q366" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R366" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -24779,14 +24779,14 @@
         <v>0</v>
       </c>
       <c r="P370" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q370" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R370" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -25051,14 +25051,14 @@
         <v>0</v>
       </c>
       <c r="P374" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q374" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R374" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -25323,10 +25323,10 @@
         <v>1</v>
       </c>
       <c r="P378" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q378" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R378" t="inlineStr">
         <is>
@@ -25799,14 +25799,14 @@
         <v>0</v>
       </c>
       <c r="P385" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q385" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R385" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -27363,10 +27363,10 @@
         <v>0</v>
       </c>
       <c r="P408" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q408" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R408" t="inlineStr">
         <is>
@@ -27907,10 +27907,10 @@
         <v>0</v>
       </c>
       <c r="P416" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q416" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R416" t="inlineStr">
         <is>
@@ -29267,10 +29267,10 @@
         <v>0</v>
       </c>
       <c r="P436" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q436" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R436" t="inlineStr">
         <is>
@@ -29539,14 +29539,14 @@
         <v>0</v>
       </c>
       <c r="P440" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q440" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R440" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -29743,14 +29743,14 @@
         <v>0</v>
       </c>
       <c r="P443" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q443" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R443" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -30899,14 +30899,14 @@
         <v>0</v>
       </c>
       <c r="P460" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q460" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R460" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -31239,14 +31239,14 @@
         <v>0</v>
       </c>
       <c r="P465" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q465" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R465" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -31783,10 +31783,10 @@
         <v>0</v>
       </c>
       <c r="P473" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q473" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R473" t="inlineStr">
         <is>
@@ -33075,14 +33075,14 @@
         <v>0</v>
       </c>
       <c r="P492" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q492" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R492" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -33211,14 +33211,14 @@
         <v>0</v>
       </c>
       <c r="P494" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q494" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R494" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -33687,14 +33687,14 @@
         <v>0</v>
       </c>
       <c r="P501" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q501" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R501" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -35863,14 +35863,14 @@
         <v>0</v>
       </c>
       <c r="P533" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q533" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R533" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -36135,14 +36135,14 @@
         <v>0</v>
       </c>
       <c r="P537" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q537" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R537" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -36611,14 +36611,14 @@
         <v>0</v>
       </c>
       <c r="P544" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q544" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R544" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -37087,14 +37087,14 @@
         <v>0</v>
       </c>
       <c r="P551" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q551" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R551" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -38243,14 +38243,14 @@
         <v>0</v>
       </c>
       <c r="P568" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q568" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R568" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -38379,14 +38379,14 @@
         <v>0</v>
       </c>
       <c r="P570" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q570" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R570" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -38719,14 +38719,14 @@
         <v>0</v>
       </c>
       <c r="P575" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q575" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R575" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -38923,14 +38923,14 @@
         <v>0</v>
       </c>
       <c r="P578" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q578" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R578" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -39603,14 +39603,14 @@
         <v>0</v>
       </c>
       <c r="P588" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q588" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R588" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -39807,14 +39807,14 @@
         <v>0</v>
       </c>
       <c r="P591" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q591" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R591" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -40827,14 +40827,14 @@
         <v>0</v>
       </c>
       <c r="P606" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q606" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R606" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -41371,14 +41371,14 @@
         <v>0</v>
       </c>
       <c r="P614" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q614" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R614" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -42051,14 +42051,14 @@
         <v>0</v>
       </c>
       <c r="P624" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q624" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R624" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -43683,14 +43683,14 @@
         <v>0</v>
       </c>
       <c r="P648" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q648" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R648" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -47287,14 +47287,14 @@
         <v>0</v>
       </c>
       <c r="P701" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q701" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R701" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -47763,14 +47763,14 @@
         <v>0</v>
       </c>
       <c r="P708" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q708" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R708" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -48511,14 +48511,14 @@
         <v>0</v>
       </c>
       <c r="P719" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q719" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R719" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -48647,14 +48647,14 @@
         <v>0</v>
       </c>
       <c r="P721" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q721" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R721" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -49803,14 +49803,14 @@
         <v>0</v>
       </c>
       <c r="P738" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q738" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R738" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -51503,14 +51503,14 @@
         <v>0</v>
       </c>
       <c r="P763" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q763" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R763" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -51775,14 +51775,14 @@
         <v>0</v>
       </c>
       <c r="P767" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q767" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R767" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -51843,14 +51843,14 @@
         <v>0</v>
       </c>
       <c r="P768" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q768" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R768" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -52659,14 +52659,14 @@
         <v>0</v>
       </c>
       <c r="P780" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q780" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R780" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -52863,14 +52863,14 @@
         <v>0</v>
       </c>
       <c r="P783" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q783" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R783" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -53135,14 +53135,14 @@
         <v>0</v>
       </c>
       <c r="P787" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q787" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R787" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -53203,14 +53203,14 @@
         <v>0</v>
       </c>
       <c r="P788" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q788" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R788" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -53815,14 +53815,14 @@
         <v>0</v>
       </c>
       <c r="P797" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q797" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R797" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -54427,14 +54427,14 @@
         <v>0</v>
       </c>
       <c r="P806" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q806" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R806" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -55039,14 +55039,14 @@
         <v>0</v>
       </c>
       <c r="P815" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q815" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R815" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -55107,14 +55107,14 @@
         <v>0</v>
       </c>
       <c r="P816" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q816" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R816" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -55175,14 +55175,14 @@
         <v>0</v>
       </c>
       <c r="P817" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q817" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R817" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -55855,14 +55855,14 @@
         <v>0</v>
       </c>
       <c r="P827" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q827" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R827" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -56875,14 +56875,14 @@
         <v>0</v>
       </c>
       <c r="P842" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q842" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R842" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -57079,14 +57079,14 @@
         <v>0</v>
       </c>
       <c r="P845" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q845" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R845" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -58711,14 +58711,14 @@
         <v>0</v>
       </c>
       <c r="P869" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q869" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R869" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -59187,14 +59187,14 @@
         <v>0</v>
       </c>
       <c r="P876" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q876" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R876" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -59799,14 +59799,14 @@
         <v>0</v>
       </c>
       <c r="P885" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q885" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R885" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -60411,14 +60411,14 @@
         <v>0</v>
       </c>
       <c r="P894" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q894" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R894" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -61227,14 +61227,14 @@
         <v>0</v>
       </c>
       <c r="P906" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q906" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R906" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -61771,14 +61771,14 @@
         <v>0</v>
       </c>
       <c r="P914" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q914" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R914" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -62995,14 +62995,14 @@
         <v>0</v>
       </c>
       <c r="P932" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q932" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R932" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -65103,14 +65103,14 @@
         <v>0</v>
       </c>
       <c r="P963" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q963" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R963" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -68707,14 +68707,14 @@
         <v>0</v>
       </c>
       <c r="P1016" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1016" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1016" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -68979,14 +68979,14 @@
         <v>0</v>
       </c>
       <c r="P1020" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1020" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1020" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -69183,14 +69183,14 @@
         <v>0</v>
       </c>
       <c r="P1023" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1023" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1023" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -70475,14 +70475,14 @@
         <v>0</v>
       </c>
       <c r="P1042" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1042" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1042" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -71223,14 +71223,14 @@
         <v>0</v>
       </c>
       <c r="P1053" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1053" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1053" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -72379,14 +72379,14 @@
         <v>0</v>
       </c>
       <c r="P1070" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1070" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1070" t="inlineStr">
         <is>
-          <t>delete-page-candidate</t>
+          <t>salvage-wayback</t>
         </is>
       </c>
     </row>
@@ -75275,10 +75275,10 @@
         <v>0</v>
       </c>
       <c r="P1113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1113" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R1113" t="inlineStr">
         <is>
@@ -80375,10 +80375,10 @@
         <v>2</v>
       </c>
       <c r="P1188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1188" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R1188" t="inlineStr">
         <is>
@@ -81395,10 +81395,10 @@
         <v>0</v>
       </c>
       <c r="P1203" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1203" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1203" t="inlineStr">
         <is>
@@ -81599,10 +81599,10 @@
         <v>0</v>
       </c>
       <c r="P1206" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1206" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add decision dropdown column to review sheet xlsx output
Both link_review_master.xlsx and link_review_pages.xlsx now end with a
blank 'decision' column carrying a data-validation dropdown (link-level:
remove / update-to-final-url / salvage-wayback / salvage-new-link / keep;
page-level: delete-page / salvage-wayback / fix-links / keep), so the
team records calls in a consistent vocabulary the future apply step can
consume. CSV outputs are unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/utils/link_review_pages.xlsx
+++ b/utils/link_review_pages.xlsx
@@ -10,7 +10,7 @@
     <sheet name="page_review" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'page_review'!$A$1:$R$1207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'page_review'!$A$1:$S$1207</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1207"/>
+  <dimension ref="A1:S1207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -440,6 +440,7 @@
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,6 +534,11 @@
           <t>suggested_page_action</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -81679,7 +81685,12 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1207"/>
+  <autoFilter ref="A1:S1207"/>
+  <dataValidations count="1">
+    <dataValidation sqref="S2:S1207" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"delete-page,salvage-wayback,fix-links,keep"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>